<commit_message>
Finished Majority Element with 2 solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="23">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t>Missing Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Majority Number </t>
   </si>
   <si>
     <t>Valid Palindrome</t>
@@ -637,21 +640,38 @@
       <c r="A13" s="4">
         <v>11.0</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="7" t="s">
+      <c r="C13" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="11">
         <v>0.0</v>
       </c>
       <c r="F13" s="5"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1"/>
+    <row r="14" ht="19.5" customHeight="1">
+      <c r="A14" s="4">
+        <v>12.0</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="F14" s="5"/>
+    </row>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1"/>
     <row r="26" ht="15.75" customHeight="1"/>
@@ -1631,6 +1651,7 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
     <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>

</xml_diff>

<commit_message>
Finished Two Sum II - Input Array Is Sorted
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="24">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -80,13 +80,16 @@
   </si>
   <si>
     <t>Two Pointers</t>
+  </si>
+  <si>
+    <t>Two Sum II Input Array Is Sorted</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -129,8 +132,17 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -141,6 +153,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F2937"/>
         <bgColor rgb="FF1F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6B8AF"/>
+        <bgColor rgb="FFE6B8AF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDD7E6B"/>
+        <bgColor rgb="FFDD7E6B"/>
       </patternFill>
     </fill>
   </fills>
@@ -164,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -183,12 +207,15 @@
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -203,12 +230,73 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00FF00"/>
+          <bgColor rgb="FF00FF00"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -469,7 +557,7 @@
       <c r="D3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="8">
         <v>0.0</v>
       </c>
       <c r="F3" s="5"/>
@@ -487,7 +575,7 @@
       <c r="D4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="8">
         <v>0.0</v>
       </c>
       <c r="F4" s="5"/>
@@ -505,7 +593,7 @@
       <c r="D5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="8">
         <v>0.0</v>
       </c>
       <c r="F5" s="5"/>
@@ -520,10 +608,10 @@
       <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="8">
         <v>0.0</v>
       </c>
       <c r="F6" s="5"/>
@@ -538,10 +626,10 @@
       <c r="C7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="8">
         <v>0.0</v>
       </c>
       <c r="F7" s="5"/>
@@ -556,10 +644,10 @@
       <c r="C8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="8">
         <v>0.0</v>
       </c>
       <c r="F8" s="5"/>
@@ -574,10 +662,10 @@
       <c r="C9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="8">
         <v>0.0</v>
       </c>
       <c r="F9" s="5"/>
@@ -592,10 +680,10 @@
       <c r="C10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="8">
         <v>0.0</v>
       </c>
       <c r="F10" s="5"/>
@@ -604,16 +692,16 @@
       <c r="A11" s="4">
         <v>9.0</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="12">
         <v>0.0</v>
       </c>
       <c r="F11" s="5"/>
@@ -622,16 +710,16 @@
       <c r="A12" s="4">
         <v>10.0</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="12">
         <v>0.0</v>
       </c>
       <c r="F12" s="5"/>
@@ -640,16 +728,16 @@
       <c r="A13" s="4">
         <v>11.0</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="12">
         <v>0.0</v>
       </c>
       <c r="F13" s="5"/>
@@ -661,18 +749,38 @@
       <c r="B14" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="15" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="8">
         <v>0.0</v>
       </c>
       <c r="F14" s="5"/>
     </row>
-    <row r="24" ht="15.75" customHeight="1"/>
+    <row r="15" ht="19.5" customHeight="1">
+      <c r="A15" s="4">
+        <v>13.0</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F15" s="20"/>
+    </row>
+    <row r="16">
+      <c r="D16" s="21"/>
+    </row>
     <row r="25" ht="15.75" customHeight="1"/>
     <row r="26" ht="15.75" customHeight="1"/>
     <row r="27" ht="15.75" customHeight="1"/>
@@ -1652,10 +1760,26 @@
     <row r="1001" ht="15.75" customHeight="1"/>
     <row r="1002" ht="15.75" customHeight="1"/>
     <row r="1003" ht="15.75" customHeight="1"/>
+    <row r="1004" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <conditionalFormatting sqref="D1:D1004">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Easy">
+      <formula>NOT(ISERROR(SEARCH(("Easy"),(D1))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:D1004">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Medium">
+      <formula>NOT(ISERROR(SEARCH(("Medium"),(D1))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:D1004">
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Hard">
+      <formula>NOT(ISERROR(SEARCH(("Hard"),(D1))))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
Finished Container with most water in 2 solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="26">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t>3Sum</t>
+  </si>
+  <si>
+    <t>Container With Most Water</t>
   </si>
 </sst>
 </file>
@@ -191,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -254,6 +257,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -799,10 +805,27 @@
       </c>
       <c r="F16" s="20"/>
     </row>
-    <row r="17">
-      <c r="D17" s="21"/>
+    <row r="17" ht="19.5" customHeight="1">
+      <c r="A17" s="4">
+        <v>15.0</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F17" s="20"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="18">
+      <c r="D18" s="22"/>
+    </row>
     <row r="27" ht="15.75" customHeight="1"/>
     <row r="28" ht="15.75" customHeight="1"/>
     <row r="29" ht="15.75" customHeight="1"/>
@@ -1782,21 +1805,22 @@
     <row r="1003" ht="15.75" customHeight="1"/>
     <row r="1004" ht="15.75" customHeight="1"/>
     <row r="1005" ht="15.75" customHeight="1"/>
+    <row r="1006" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D1:D1005">
+  <conditionalFormatting sqref="D1:D1006">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Easy">
       <formula>NOT(ISERROR(SEARCH(("Easy"),(D1))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:D1005">
+  <conditionalFormatting sqref="D1:D1006">
     <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH(("Medium"),(D1))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:D1005">
+  <conditionalFormatting sqref="D1:D1006">
     <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Hard">
       <formula>NOT(ISERROR(SEARCH(("Hard"),(D1))))</formula>
     </cfRule>

</xml_diff>

<commit_message>
Finished Trapping Rain water in 2 solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="28">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -89,13 +89,19 @@
   </si>
   <si>
     <t>Container With Most Water</t>
+  </si>
+  <si>
+    <t>Trapping Rain Water</t>
+  </si>
+  <si>
+    <t>Hard</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -141,6 +147,12 @@
     <font>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
@@ -194,7 +206,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -262,7 +274,10 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -824,7 +839,21 @@
       <c r="F17" s="20"/>
     </row>
     <row r="18">
-      <c r="D18" s="22"/>
+      <c r="A18" s="4">
+        <v>16.0</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="23">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1"/>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Finished Squares of Sorted Array in 4 solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="30">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -98,6 +98,9 @@
   </si>
   <si>
     <t xml:space="preserve">Move Zeroes </t>
+  </si>
+  <si>
+    <t>Squares of Sorted Array</t>
   </si>
 </sst>
 </file>
@@ -200,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -251,9 +254,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
@@ -1042,16 +1042,16 @@
       <c r="B15" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="17" t="s">
         <v>13</v>
       </c>
       <c r="E15" s="6">
         <v>0.0</v>
       </c>
-      <c r="F15" s="19"/>
+      <c r="F15" s="18"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -1079,16 +1079,16 @@
       <c r="B16" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="17" t="s">
         <v>13</v>
       </c>
       <c r="E16" s="6">
         <v>0.0</v>
       </c>
-      <c r="F16" s="19"/>
+      <c r="F16" s="18"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -1113,19 +1113,19 @@
       <c r="A17" s="6">
         <v>15.0</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="17" t="s">
         <v>13</v>
       </c>
       <c r="E17" s="6">
         <v>0.0</v>
       </c>
-      <c r="F17" s="19"/>
+      <c r="F17" s="18"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -1153,7 +1153,7 @@
       <c r="B18" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="15" t="s">
         <v>22</v>
       </c>
       <c r="D18" s="16" t="s">
@@ -1190,7 +1190,7 @@
       <c r="B19" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="15" t="s">
         <v>22</v>
       </c>
       <c r="D19" s="16" t="s">
@@ -1221,11 +1221,21 @@
       <c r="Y19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
+      <c r="A20" s="16">
+        <v>18.0</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" s="16">
+        <v>0.0</v>
+      </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>

</xml_diff>

<commit_message>
Finished Best Time to Buy and Sell Stock in one solution
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="35">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -58,10 +58,16 @@
     <t>Top K Frequent Elements</t>
   </si>
   <si>
+    <t xml:space="preserve">Make sure to remember the algorithm </t>
+  </si>
+  <si>
     <t>Product of Array Except Self</t>
   </si>
   <si>
     <t>Valid Sudoku</t>
+  </si>
+  <si>
+    <t>This needs care</t>
   </si>
   <si>
     <t>Longest Consecutive Sequence</t>
@@ -101,6 +107,15 @@
   </si>
   <si>
     <t>Squares of Sorted Array</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best Time to Buy and Sell Stock </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sliding Window </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Easy </t>
   </si>
 </sst>
 </file>
@@ -157,7 +172,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -182,6 +197,12 @@
         <bgColor rgb="FFDD7E6B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9CB9C"/>
+        <bgColor rgb="FFF9CB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -203,7 +224,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -262,6 +283,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -523,7 +547,7 @@
     <col customWidth="1" min="3" max="3" width="31.86"/>
     <col customWidth="1" min="4" max="4" width="26.0"/>
     <col customWidth="1" min="5" max="5" width="29.0"/>
-    <col customWidth="1" min="6" max="6" width="30.0"/>
+    <col customWidth="1" min="6" max="6" width="36.57"/>
     <col customWidth="1" min="7" max="25" width="8.71"/>
   </cols>
   <sheetData>
@@ -755,7 +779,9 @@
       <c r="E7" s="7">
         <v>0.0</v>
       </c>
-      <c r="F7" s="7"/>
+      <c r="F7" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -781,7 +807,7 @@
         <v>6.0</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>8</v>
@@ -818,7 +844,7 @@
         <v>7.0</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>8</v>
@@ -829,7 +855,9 @@
       <c r="E9" s="7">
         <v>0.0</v>
       </c>
-      <c r="F9" s="7"/>
+      <c r="F9" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -855,7 +883,7 @@
         <v>8.0</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>8</v>
@@ -892,7 +920,7 @@
         <v>9.0</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>8</v>
@@ -929,7 +957,7 @@
         <v>10.0</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C12" s="14" t="s">
         <v>8</v>
@@ -966,7 +994,7 @@
         <v>11.0</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C13" s="14" t="s">
         <v>8</v>
@@ -1003,10 +1031,10 @@
         <v>12.0</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>9</v>
@@ -1040,10 +1068,10 @@
         <v>13.0</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D15" s="17" t="s">
         <v>13</v>
@@ -1077,10 +1105,10 @@
         <v>14.0</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D16" s="17" t="s">
         <v>13</v>
@@ -1114,10 +1142,10 @@
         <v>15.0</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D17" s="17" t="s">
         <v>13</v>
@@ -1151,13 +1179,13 @@
         <v>16.0</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E18" s="16">
         <v>0.0</v>
@@ -1188,10 +1216,10 @@
         <v>17.0</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D19" s="16" t="s">
         <v>9</v>
@@ -1225,10 +1253,10 @@
         <v>18.0</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D20" s="16" t="s">
         <v>9</v>
@@ -1258,11 +1286,21 @@
       <c r="Y20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+      <c r="A21" s="16">
+        <v>19.0</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="16">
+        <v>0.0</v>
+      </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>

</xml_diff>

<commit_message>
Finished Longest Substring Without Repeating Characters in one solution
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="37">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -117,12 +117,18 @@
   <si>
     <t xml:space="preserve">Easy </t>
   </si>
+  <si>
+    <t>Longest Substring Without Repeating Characters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sounds simple but missed out on the core sliding logic so repeat more </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -170,6 +176,11 @@
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FFFFA116"/>
+      <name val="-apple-system"/>
     </font>
   </fonts>
   <fills count="6">
@@ -224,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -287,6 +298,12 @@
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -547,7 +564,7 @@
     <col customWidth="1" min="3" max="3" width="31.86"/>
     <col customWidth="1" min="4" max="4" width="26.0"/>
     <col customWidth="1" min="5" max="5" width="29.0"/>
-    <col customWidth="1" min="6" max="6" width="36.57"/>
+    <col customWidth="1" min="6" max="6" width="66.71"/>
     <col customWidth="1" min="7" max="25" width="8.71"/>
   </cols>
   <sheetData>
@@ -1323,12 +1340,24 @@
       <c r="Y21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
+      <c r="A22" s="16">
+        <v>20.0</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="16">
+        <v>0.0</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>36</v>
+      </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
@@ -1351,7 +1380,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
+      <c r="B23" s="22"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>

</xml_diff>

<commit_message>
Finished Longest Repeating Character Replacement
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -123,12 +123,18 @@
   <si>
     <t xml:space="preserve">Sounds simple but missed out on the core sliding logic so repeat more </t>
   </si>
+  <si>
+    <t>Longest Repeating Character Replacement</t>
+  </si>
+  <si>
+    <t>Needs lot of work dude!</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -176,11 +182,6 @@
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FFFFA116"/>
-      <name val="-apple-system"/>
     </font>
   </fonts>
   <fills count="6">
@@ -235,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -301,9 +302,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1379,12 +1377,24 @@
       <c r="Y22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="2"/>
-      <c r="B23" s="22"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
+      <c r="A23" s="16">
+        <v>21.0</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" s="16">
+        <v>0.0</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>38</v>
+      </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>

</xml_diff>

<commit_message>
Finished Permutation in String in one solution
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="40">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -128,6 +128,9 @@
   </si>
   <si>
     <t>Needs lot of work dude!</t>
+  </si>
+  <si>
+    <t>Permutation In String</t>
   </si>
 </sst>
 </file>
@@ -1416,11 +1419,21 @@
       <c r="Y23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
+      <c r="A24" s="16">
+        <v>22.0</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" s="16">
+        <v>0.0</v>
+      </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>

</xml_diff>

<commit_message>
Finished Minimum Window Substring with 2 solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="42">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -131,6 +131,12 @@
   </si>
   <si>
     <t>Permutation In String</t>
+  </si>
+  <si>
+    <t>Minimum Window Substring</t>
+  </si>
+  <si>
+    <t>Needs a lot of work dude!</t>
   </si>
 </sst>
 </file>
@@ -1456,12 +1462,24 @@
       <c r="Y24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
+      <c r="A25" s="16">
+        <v>23.0</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25" s="16">
+        <v>0.0</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>41</v>
+      </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>

</xml_diff>

<commit_message>
Finished Sliding Window Maximum in two solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="44">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -138,12 +138,18 @@
   <si>
     <t>Needs a lot of work dude!</t>
   </si>
+  <si>
+    <t>Sliding Window Maximum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seems like a simple problem if bruteforced, but must use queue for an optimal solution </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -191,6 +197,11 @@
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -245,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -310,6 +321,9 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -571,7 +585,7 @@
     <col customWidth="1" min="3" max="3" width="31.86"/>
     <col customWidth="1" min="4" max="4" width="26.0"/>
     <col customWidth="1" min="5" max="5" width="29.0"/>
-    <col customWidth="1" min="6" max="6" width="66.71"/>
+    <col customWidth="1" min="6" max="6" width="81.86"/>
     <col customWidth="1" min="7" max="25" width="8.71"/>
   </cols>
   <sheetData>
@@ -1501,12 +1515,24 @@
       <c r="Y25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
+      <c r="A26" s="16">
+        <v>24.0</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" s="16">
+        <v>0.0</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>43</v>
+      </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>

</xml_diff>

<commit_message>
4 Problems Revision + Group Anagrams another solution + Code refactor to follow the right programming methods of all files
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -287,11 +287,11 @@
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
@@ -666,8 +666,8 @@
       <c r="D3" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="7">
-        <v>0.0</v>
+      <c r="E3" s="10">
+        <v>2.0</v>
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="2"/>
@@ -703,8 +703,8 @@
       <c r="D4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="7">
-        <v>0.0</v>
+      <c r="E4" s="10">
+        <v>2.0</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="2"/>
@@ -740,8 +740,8 @@
       <c r="D5" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="7">
-        <v>0.0</v>
+      <c r="E5" s="10">
+        <v>1.0</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="2"/>
@@ -774,11 +774,11 @@
       <c r="C6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="7">
-        <v>0.0</v>
+      <c r="E6" s="10">
+        <v>1.0</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="2"/>
@@ -811,13 +811,13 @@
       <c r="C7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="7">
         <v>0.0</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="10" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="2"/>
@@ -850,7 +850,7 @@
       <c r="C8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E8" s="7">
@@ -887,13 +887,13 @@
       <c r="C9" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E9" s="7">
         <v>0.0</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="10" t="s">
         <v>18</v>
       </c>
       <c r="G9" s="2"/>
@@ -926,7 +926,7 @@
       <c r="C10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E10" s="7">
@@ -957,7 +957,7 @@
       <c r="A11" s="6">
         <v>9.0</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="8" t="s">
@@ -966,7 +966,7 @@
       <c r="D11" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="10">
         <v>0.0</v>
       </c>
       <c r="F11" s="7"/>
@@ -1003,7 +1003,7 @@
       <c r="D12" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="10">
         <v>0.0</v>
       </c>
       <c r="F12" s="7"/>
@@ -1040,7 +1040,7 @@
       <c r="D13" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="10">
         <v>0.0</v>
       </c>
       <c r="F13" s="7"/>

</xml_diff>

<commit_message>
Revised one problem, but should def speed up
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -58,7 +58,7 @@
     <t>Top K Frequent Elements</t>
   </si>
   <si>
-    <t xml:space="preserve">Make sure to remember the algorithm </t>
+    <t>Make sure to remember the algorithm , Revise more!! basically map sorting syntax based on values!!!</t>
   </si>
   <si>
     <t>Product of Array Except Self</t>
@@ -585,7 +585,7 @@
     <col customWidth="1" min="3" max="3" width="31.86"/>
     <col customWidth="1" min="4" max="4" width="26.0"/>
     <col customWidth="1" min="5" max="5" width="29.0"/>
-    <col customWidth="1" min="6" max="6" width="81.86"/>
+    <col customWidth="1" min="6" max="6" width="95.0"/>
     <col customWidth="1" min="7" max="25" width="8.71"/>
   </cols>
   <sheetData>
@@ -814,8 +814,8 @@
       <c r="D7" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="7">
-        <v>0.0</v>
+      <c r="E7" s="10">
+        <v>1.0</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Finished Valid Parenthses in 2 solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="46">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -144,6 +144,12 @@
   <si>
     <t xml:space="preserve">Seems like a simple problem if bruteforced, but must use queue for an optimal solution </t>
   </si>
+  <si>
+    <t>Valid Parentheses</t>
+  </si>
+  <si>
+    <t>Stack</t>
+  </si>
 </sst>
 </file>
 
@@ -204,7 +210,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -235,6 +241,12 @@
         <bgColor rgb="FFF9CB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF93C47D"/>
+        <bgColor rgb="FF93C47D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -256,7 +268,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -325,6 +337,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1554,11 +1569,21 @@
       <c r="Y26" s="2"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
+      <c r="A27" s="16">
+        <v>25.0</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="16">
+        <v>0.0</v>
+      </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>

</xml_diff>

<commit_message>
Finished Binary Search in 2 solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="47">
   <si>
     <t>LeetCode Revision Tracker</t>
   </si>
@@ -150,6 +150,9 @@
   <si>
     <t>Stack</t>
   </si>
+  <si>
+    <t>Binary Search</t>
+  </si>
 </sst>
 </file>
 
@@ -210,7 +213,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -247,6 +250,12 @@
         <bgColor rgb="FF93C47D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6D9EEB"/>
+        <bgColor rgb="FF6D9EEB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -268,7 +277,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -339,6 +348,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -1606,11 +1618,21 @@
       <c r="Y27" s="2"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
+      <c r="A28" s="16">
+        <v>26.0</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28" s="16">
+        <v>0.0</v>
+      </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>

</xml_diff>

<commit_message>
Finished Linked List cycle
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="52">
   <si>
     <t>LeetCode Revision Tracker - Neetcode 150</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t>Linked List</t>
+  </si>
+  <si>
+    <t>Linked LIst cycle</t>
   </si>
 </sst>
 </file>
@@ -799,7 +802,7 @@
       </c>
       <c r="F2" s="5" t="str">
         <f>"Did I Solve on my own?  Self solved: ("&amp;TEXT(COUNTIF(F3:F1000,"Yes")/COUNTIF(F3:F1000,"&lt;&gt;")*100,"0")&amp;"%)"</f>
-        <v>Did I Solve on my own?  Self solved: (52%)</v>
+        <v>Did I Solve on my own?  Self solved: (50%)</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>6</v>
@@ -1920,11 +1923,21 @@
       <c r="A30" s="17">
         <v>28.0</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
+      <c r="B30" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30" s="17">
+        <v>0.0</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>15</v>
+      </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
       <c r="I30" s="6"/>

</xml_diff>

<commit_message>
Finished Minstack with 3 solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="53">
   <si>
     <t>LeetCode Revision Tracker - Neetcode 150</t>
   </si>
@@ -167,6 +167,9 @@
   </si>
   <si>
     <t>Linked LIst cycle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min Stack </t>
   </si>
 </sst>
 </file>
@@ -802,7 +805,7 @@
       </c>
       <c r="F2" s="5" t="str">
         <f>"Did I Solve on my own?  Self solved: ("&amp;TEXT(COUNTIF(F3:F1000,"Yes")/COUNTIF(F3:F1000,"&lt;&gt;")*100,"0")&amp;"%)"</f>
-        <v>Did I Solve on my own?  Self solved: (50%)</v>
+        <v>Did I Solve on my own?  Self solved: (48%)</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>6</v>
@@ -1963,11 +1966,21 @@
       <c r="A31" s="17">
         <v>29.0</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
+      <c r="B31" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" s="17">
+        <v>0.0</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>15</v>
+      </c>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
@@ -29576,8 +29589,8 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C1006">
-    <cfRule type="containsText" dxfId="8" priority="9" operator="containsText" text="Stack ">
-      <formula>NOT(ISERROR(SEARCH(("Stack "),(C2))))</formula>
+    <cfRule type="containsText" dxfId="8" priority="9" operator="containsText" text="Stack">
+      <formula>NOT(ISERROR(SEARCH(("Stack"),(C2))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C1006">

</xml_diff>

<commit_message>
Finished Car Fleet in 2 solutions
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="60">
   <si>
     <t>LeetCode Revision Tracker - Neetcode 150</t>
   </si>
@@ -189,6 +189,9 @@
   <si>
     <t>Daily Temperatures</t>
   </si>
+  <si>
+    <t>Car Fleet</t>
+  </si>
 </sst>
 </file>
 
@@ -336,7 +339,7 @@
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -345,16 +348,16 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -390,7 +393,7 @@
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -855,7 +858,7 @@
       </c>
       <c r="F2" s="6" t="str">
         <f>"Did I Solve on my own?  Self solved: ("&amp;TEXT(COUNTIF(F3:F1000,"Yes")/COUNTIF(F3:F1000,"&lt;&gt;")*100,"0")&amp;"%)"</f>
-        <v>Did I Solve on my own?  Self solved: (48%)</v>
+        <v>Did I Solve on my own?  Self solved: (47%)</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>6</v>
@@ -2520,16 +2523,34 @@
       <c r="A34" s="22">
         <v>32.0</v>
       </c>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="34"/>
-      <c r="H34" s="34"/>
-      <c r="I34" s="34"/>
+      <c r="B34" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="D34" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" s="22">
+        <v>0.0</v>
+      </c>
+      <c r="F34" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="G34" s="26">
+        <v>46262.89674409722</v>
+      </c>
+      <c r="H34" s="26">
+        <v>46269.89674409722</v>
+      </c>
+      <c r="I34" s="26">
+        <v>46283.89674409722</v>
+      </c>
       <c r="J34" s="9"/>
-      <c r="K34" s="34"/>
+      <c r="K34" s="26">
+        <v>46255.89674409722</v>
+      </c>
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9"/>

</xml_diff>

<commit_message>
Finished Largest Rectangle in Histogram
</commit_message>
<xml_diff>
--- a/Leetcode_tracker.xlsx
+++ b/Leetcode_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="62">
   <si>
     <t>LeetCode Revision Tracker - Neetcode 150</t>
   </si>
@@ -191,6 +191,12 @@
   </si>
   <si>
     <t>Car Fleet</t>
+  </si>
+  <si>
+    <t>Largest Rectangle in Histogram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stack </t>
   </si>
 </sst>
 </file>
@@ -858,7 +864,7 @@
       </c>
       <c r="F2" s="6" t="str">
         <f>"Did I Solve on my own?  Self solved: ("&amp;TEXT(COUNTIF(F3:F1000,"Yes")/COUNTIF(F3:F1000,"&lt;&gt;")*100,"0")&amp;"%)"</f>
-        <v>Did I Solve on my own?  Self solved: (47%)</v>
+        <v>Did I Solve on my own?  Self solved: (45%)</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>6</v>
@@ -2575,16 +2581,34 @@
       <c r="A35" s="22">
         <v>33.0</v>
       </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="34"/>
-      <c r="I35" s="34"/>
+      <c r="B35" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="D35" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="E35" s="22">
+        <v>0.0</v>
+      </c>
+      <c r="F35" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="26">
+        <v>46266.04734615741</v>
+      </c>
+      <c r="H35" s="26">
+        <v>46273.04734615741</v>
+      </c>
+      <c r="I35" s="26">
+        <v>46287.04734615741</v>
+      </c>
       <c r="J35" s="9"/>
-      <c r="K35" s="34"/>
+      <c r="K35" s="26">
+        <v>46259.04734615741</v>
+      </c>
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9"/>

</xml_diff>